<commit_message>
yay i can go sleep now
ill be sleeping well
</commit_message>
<xml_diff>
--- a/Физика варианты 11-7 (2025_26).xlsx
+++ b/Физика варианты 11-7 (2025_26).xlsx
@@ -1961,10 +1961,10 @@
         <v>1</v>
       </c>
       <c r="F11" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" s="31" t="n">
         <v>0</v>
@@ -5727,58 +5727,58 @@
         <v>0</v>
       </c>
       <c r="G4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" s="31" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V4" s="31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X4" s="31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y4" s="5" t="n">
         <v>3</v>

</xml_diff>